<commit_message>
Fix missing chart labels in sales report
The previous style_chart helper only hid gridlines and legend; it never
explicitly enabled axis tick labels, set chart titles, formatted value
axes, or surfaced data labels, so the charts rendered as bare lines and
bars in some viewers. Now both charts get a title, axis.delete=False is
set explicitly, the value axis is formatted in millions of won (백만원),
and the regional bar chart shows per-bar value labels. The line chart
also gets red circle markers at each monthly point.

Two correctness fixes folded in:
- chart_text() was emitting <a:r><a:t /></a:r> because openpyxl's
  Paragraph defaults r to a single empty RegularTextRun; pass r=[] so
  the txPr block contains only pPr/endParaRPr as the schema expects.
- numFmt was being applied to chart.x_axis (CategoryAxis) for horizontal
  bars, which is incorrect — chart.y_axis is always the ValueAxis in
  openpyxl regardless of bar orientation.
</commit_message>
<xml_diff>
--- a/엑셀 파일 튜토리얼/sales_report.xlsx
+++ b/엑셀 파일 튜토리얼/sales_report.xlsx
@@ -279,6 +279,21 @@
 <file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
 <chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
+    <title>
+      <tx>
+        <rich>
+          <a:bodyPr/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:t>월별 매출 (단위: 백만원)</a:t>
+            </a:r>
+          </a:p>
+        </rich>
+      </tx>
+    </title>
     <plotArea>
       <lineChart>
         <grouping val="standard"/>
@@ -299,9 +314,16 @@
             </a:ln>
           </spPr>
           <marker>
-            <symbol val="none"/>
+            <symbol val="circle"/>
+            <size val="6"/>
             <spPr>
+              <a:solidFill>
+                <a:srgbClr val="A50034"/>
+              </a:solidFill>
               <a:ln>
+                <a:solidFill>
+                  <a:srgbClr val="A50034"/>
+                </a:solidFill>
                 <a:prstDash val="solid"/>
               </a:ln>
             </spPr>
@@ -316,6 +338,7 @@
               <f>'분석 결과'!$C$9:$C$20</f>
             </numRef>
           </val>
+          <smooth val="0"/>
         </ser>
         <axId val="10"/>
         <axId val="100"/>
@@ -325,9 +348,29 @@
         <scaling>
           <orientation val="minMax"/>
         </scaling>
+        <delete val="0"/>
         <axPos val="l"/>
         <majorTickMark val="none"/>
         <minorTickMark val="none"/>
+        <txPr>
+          <a:bodyPr/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0">
+                <a:solidFill>
+                  <a:srgbClr val="6B6B6B"/>
+                </a:solidFill>
+                <a:latin typeface="Calibri"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr sz="900" b="0">
+              <a:solidFill>
+                <a:srgbClr val="6B6B6B"/>
+              </a:solidFill>
+              <a:latin typeface="Calibri"/>
+            </a:endParaRPr>
+          </a:p>
+        </txPr>
         <crossAx val="100"/>
         <lblOffset val="100"/>
       </catAx>
@@ -336,9 +379,30 @@
         <scaling>
           <orientation val="minMax"/>
         </scaling>
+        <delete val="0"/>
         <axPos val="l"/>
+        <numFmt formatCode="#,##0,,&quot;M&quot;" sourceLinked="0"/>
         <majorTickMark val="none"/>
         <minorTickMark val="none"/>
+        <txPr>
+          <a:bodyPr/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0">
+                <a:solidFill>
+                  <a:srgbClr val="6B6B6B"/>
+                </a:solidFill>
+                <a:latin typeface="Calibri"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr sz="900" b="0">
+              <a:solidFill>
+                <a:srgbClr val="6B6B6B"/>
+              </a:solidFill>
+              <a:latin typeface="Calibri"/>
+            </a:endParaRPr>
+          </a:p>
+        </txPr>
         <crossAx val="10"/>
       </valAx>
     </plotArea>
@@ -352,6 +416,21 @@
 <chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <style val="2"/>
   <chart>
+    <title>
+      <tx>
+        <rich>
+          <a:bodyPr/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:t>지역별 매출 (단위: 백만원)</a:t>
+            </a:r>
+          </a:p>
+        </rich>
+      </tx>
+    </title>
     <plotArea>
       <barChart>
         <barDir val="bar"/>
@@ -386,6 +465,32 @@
             </numRef>
           </val>
         </ser>
+        <dLbls>
+          <numFmt formatCode="#,##0,,&quot;M&quot;"/>
+          <txPr>
+            <a:bodyPr/>
+            <a:p>
+              <a:pPr>
+                <a:defRPr sz="800" b="0">
+                  <a:solidFill>
+                    <a:srgbClr val="6B6B6B"/>
+                  </a:solidFill>
+                  <a:latin typeface="Calibri"/>
+                </a:defRPr>
+              </a:pPr>
+              <a:endParaRPr sz="800" b="0">
+                <a:solidFill>
+                  <a:srgbClr val="6B6B6B"/>
+                </a:solidFill>
+                <a:latin typeface="Calibri"/>
+              </a:endParaRPr>
+            </a:p>
+          </txPr>
+          <showLegendKey val="0"/>
+          <showVal val="1"/>
+          <showCatName val="0"/>
+          <showSerName val="0"/>
+        </dLbls>
         <gapWidth val="150"/>
         <axId val="10"/>
         <axId val="100"/>
@@ -395,9 +500,29 @@
         <scaling>
           <orientation val="minMax"/>
         </scaling>
+        <delete val="0"/>
         <axPos val="l"/>
         <majorTickMark val="none"/>
         <minorTickMark val="none"/>
+        <txPr>
+          <a:bodyPr/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0">
+                <a:solidFill>
+                  <a:srgbClr val="6B6B6B"/>
+                </a:solidFill>
+                <a:latin typeface="Calibri"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr sz="900" b="0">
+              <a:solidFill>
+                <a:srgbClr val="6B6B6B"/>
+              </a:solidFill>
+              <a:latin typeface="Calibri"/>
+            </a:endParaRPr>
+          </a:p>
+        </txPr>
         <crossAx val="100"/>
         <lblOffset val="100"/>
       </catAx>
@@ -406,9 +531,30 @@
         <scaling>
           <orientation val="minMax"/>
         </scaling>
+        <delete val="0"/>
         <axPos val="l"/>
+        <numFmt formatCode="#,##0,,&quot;M&quot;" sourceLinked="0"/>
         <majorTickMark val="none"/>
         <minorTickMark val="none"/>
+        <txPr>
+          <a:bodyPr/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0">
+                <a:solidFill>
+                  <a:srgbClr val="6B6B6B"/>
+                </a:solidFill>
+                <a:latin typeface="Calibri"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr sz="900" b="0">
+              <a:solidFill>
+                <a:srgbClr val="6B6B6B"/>
+              </a:solidFill>
+              <a:latin typeface="Calibri"/>
+            </a:endParaRPr>
+          </a:p>
+        </txPr>
         <crossAx val="10"/>
       </valAx>
     </plotArea>
@@ -427,7 +573,7 @@
       <row>4</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="6120000" cy="2880000"/>
+    <ext cx="6480000" cy="3240000"/>
     <graphicFrame>
       <nvGraphicFramePr>
         <cNvPr id="1" name="Chart 1"/>
@@ -449,7 +595,7 @@
       <row>23</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="6120000" cy="2880000"/>
+    <ext cx="6480000" cy="3240000"/>
     <graphicFrame>
       <nvGraphicFramePr>
         <cNvPr id="2" name="Chart 2"/>

</xml_diff>